<commit_message>
feat: implement prescriptive resource allocation engine and pipeline dashboard
</commit_message>
<xml_diff>
--- a/imports/Schedule_List_30 Connolly Ave, Coburg - FC.xlsx
+++ b/imports/Schedule_List_30 Connolly Ave, Coburg - FC.xlsx
@@ -464,118 +464,130 @@
     <t xml:space="preserve">Cladding - Installation Weathertex</t>
   </si>
   <si>
+    <t xml:space="preserve">Install of Window Glass (WEEK OF)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">84</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Internal lockup - walls</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Plaster Metal Battens + Patch Ups</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Plastering</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Oliver Trifunovski, VLS Plastering</t>
+  </si>
+  <si>
+    <t xml:space="preserve">20</t>
+  </si>
+  <si>
     <t xml:space="preserve">85</t>
   </si>
   <si>
-    <t xml:space="preserve">-3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Install of Window Glass (WEEK OF)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Internal lockup - walls</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Plaster Metal Battens + Patch Ups</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Plastering</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Oliver Trifunovski, VLS Plastering</t>
-  </si>
-  <si>
-    <t xml:space="preserve">20</t>
+    <t xml:space="preserve">3D Walkthrough</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Greg Paull, Oliver Trifunovski, Tavis King</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Flooring Installation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Floor Coverings</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Painting Exterior</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Painter</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MS Paterson Painting and Decorating, Oliver Trifunovski</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Plastering &amp; Internal Walls</t>
+  </si>
+  <si>
+    <t xml:space="preserve">88</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Carpentry Fix </t>
+  </si>
+  <si>
+    <t xml:space="preserve">89</t>
   </si>
   <si>
     <t xml:space="preserve">Decking boards</t>
   </si>
   <si>
-    <t xml:space="preserve">3D Walkthrough</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Greg Paull, Oliver Trifunovski, Tavis King</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Painting Exterior</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Painter</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MS Paterson Painting and Decorating, Oliver Trifunovski</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Plastering &amp; Internal Walls</t>
-  </si>
-  <si>
-    <t xml:space="preserve">89</t>
+    <t xml:space="preserve">Cabinetry Installation, Benchtop Templates</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Joinery</t>
+  </si>
+  <si>
+    <t xml:space="preserve">91</t>
   </si>
   <si>
     <t xml:space="preserve">Painting Interior</t>
   </si>
   <si>
-    <t xml:space="preserve">Flooring Installation</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Floor Coverings</t>
-  </si>
-  <si>
-    <t xml:space="preserve">91</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Carpentry Fix </t>
-  </si>
-  <si>
-    <t xml:space="preserve">93</t>
+    <t xml:space="preserve">92</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Benchtops - Installation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">94</t>
+  </si>
+  <si>
+    <t xml:space="preserve">9</t>
   </si>
   <si>
     <t xml:space="preserve">Carpentry Fitoff</t>
   </si>
   <si>
-    <t xml:space="preserve">92</t>
+    <t xml:space="preserve">95</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Electrical Fit Off</t>
   </si>
   <si>
     <t xml:space="preserve">Heating and Cooling - Fitoff</t>
   </si>
   <si>
-    <t xml:space="preserve">Cabinetry Installation, Benchtop Templates</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Joinery</t>
-  </si>
-  <si>
     <t xml:space="preserve">Plumbing Fitoff</t>
   </si>
   <si>
+    <t xml:space="preserve">Tiling (Splashbacks)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tiler</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Expo Marble &amp; Tiling, Oliver Trifunovski</t>
+  </si>
+  <si>
+    <t xml:space="preserve">96</t>
+  </si>
+  <si>
     <t xml:space="preserve">Site Clean - pre floor finishes</t>
   </si>
   <si>
-    <t xml:space="preserve">98</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Electrical Fit Off</t>
-  </si>
-  <si>
     <t xml:space="preserve">Floorboards - Polish</t>
   </si>
   <si>
-    <t xml:space="preserve">99</t>
+    <t xml:space="preserve">102</t>
   </si>
   <si>
     <t xml:space="preserve">Final Inspection</t>
   </si>
   <si>
-    <t xml:space="preserve">101</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Benchtops - Installation</t>
-  </si>
-  <si>
-    <t xml:space="preserve">97</t>
-  </si>
-  <si>
-    <t xml:space="preserve">9</t>
+    <t xml:space="preserve">103</t>
   </si>
   <si>
     <t xml:space="preserve">Final Certification Process</t>
@@ -584,28 +596,16 @@
     <t xml:space="preserve">Finishing &amp; Handover </t>
   </si>
   <si>
-    <t xml:space="preserve">102</t>
+    <t xml:space="preserve">104</t>
   </si>
   <si>
     <t xml:space="preserve">Final Clean</t>
   </si>
   <si>
-    <t xml:space="preserve">Tiling (Splashbacks)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tiler</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Expo Marble &amp; Tiling, Oliver Trifunovski</t>
-  </si>
-  <si>
-    <t xml:space="preserve">103</t>
-  </si>
-  <si>
     <t xml:space="preserve">Final Certificate </t>
   </si>
   <si>
-    <t xml:space="preserve">104</t>
+    <t xml:space="preserve">105</t>
   </si>
   <si>
     <t xml:space="preserve">Completion of outstanding Items</t>
@@ -620,7 +620,7 @@
     <t xml:space="preserve">Handover</t>
   </si>
   <si>
-    <t xml:space="preserve">Schedule - List - 30 Connolly Ave, Coburg - FC (exported on May 13, 2026)</t>
+    <t xml:space="preserve">Schedule - List - 30 Connolly Ave, Coburg - FC (exported on May 14, 2026)</t>
   </si>
 </sst>
 </file>
@@ -4817,15 +4817,9 @@
       <c r="L86" s="5">
         <v>0</v>
       </c>
-      <c r="M86" s="9">
-        <v>85</v>
-      </c>
-      <c r="N86" s="5" t="s">
-        <v>32</v>
-      </c>
-      <c r="O86" s="9">
-        <v>-3</v>
-      </c>
+      <c r="M86" s="0"/>
+      <c r="N86" s="0"/>
+      <c r="O86" s="0"/>
       <c r="P86" s="0"/>
       <c r="Q86" s="0"/>
       <c r="R86" s="0"/>
@@ -4838,7 +4832,7 @@
         <v>85</v>
       </c>
       <c r="B87" s="5" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="C87" s="5" t="b">
         <v>0</v>
@@ -4866,9 +4860,15 @@
       <c r="L87" s="5">
         <v>0</v>
       </c>
-      <c r="M87" s="0"/>
-      <c r="N87" s="0"/>
-      <c r="O87" s="0"/>
+      <c r="M87" s="9">
+        <v>84</v>
+      </c>
+      <c r="N87" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="O87" s="9">
+        <v>0</v>
+      </c>
       <c r="P87" s="0"/>
       <c r="Q87" s="0"/>
       <c r="R87" s="0"/>
@@ -4881,7 +4881,7 @@
         <v>86</v>
       </c>
       <c r="B88" s="5" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="C88" s="5" t="b">
         <v>0</v>
@@ -4924,16 +4924,16 @@
         <v>87</v>
       </c>
       <c r="B89" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="C89" s="5" t="b">
+        <v>0</v>
+      </c>
+      <c r="D89" s="9">
+        <v>0</v>
+      </c>
+      <c r="E89" s="5" t="s">
         <v>154</v>
-      </c>
-      <c r="C89" s="5" t="b">
-        <v>0</v>
-      </c>
-      <c r="D89" s="9">
-        <v>0</v>
-      </c>
-      <c r="E89" s="5" t="s">
-        <v>155</v>
       </c>
       <c r="F89" s="5">
         <v>2</v>
@@ -4945,7 +4945,7 @@
         <v>46168</v>
       </c>
       <c r="I89" s="5" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="J89" s="5">
         <v>0</v>
@@ -4991,17 +4991,21 @@
       <c r="D90" s="9">
         <v>0</v>
       </c>
-      <c r="E90" s="0"/>
+      <c r="E90" s="5" t="s">
+        <v>57</v>
+      </c>
       <c r="F90" s="5">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G90" s="11">
-        <v>46168</v>
+        <v>46169</v>
       </c>
       <c r="H90" s="11">
-        <v>46171</v>
-      </c>
-      <c r="I90" s="0"/>
+        <v>46169</v>
+      </c>
+      <c r="I90" s="5" t="s">
+        <v>159</v>
+      </c>
       <c r="J90" s="5">
         <v>0</v>
       </c>
@@ -5011,15 +5015,9 @@
       <c r="L90" s="5">
         <v>0</v>
       </c>
-      <c r="M90" s="9">
-        <v>85</v>
-      </c>
-      <c r="N90" s="5" t="s">
-        <v>32</v>
-      </c>
-      <c r="O90" s="9">
-        <v>1</v>
-      </c>
+      <c r="M90" s="0"/>
+      <c r="N90" s="0"/>
+      <c r="O90" s="0"/>
       <c r="P90" s="0"/>
       <c r="Q90" s="0"/>
       <c r="R90" s="0"/>
@@ -5032,7 +5030,7 @@
         <v>89</v>
       </c>
       <c r="B91" s="5" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="C91" s="5" t="b">
         <v>0</v>
@@ -5041,19 +5039,19 @@
         <v>0</v>
       </c>
       <c r="E91" s="5" t="s">
-        <v>57</v>
+        <v>161</v>
       </c>
       <c r="F91" s="5">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G91" s="11">
         <v>46169</v>
       </c>
       <c r="H91" s="11">
-        <v>46169</v>
+        <v>46171</v>
       </c>
       <c r="I91" s="5" t="s">
-        <v>160</v>
+        <v>24</v>
       </c>
       <c r="J91" s="5">
         <v>0</v>
@@ -5079,7 +5077,7 @@
         <v>90</v>
       </c>
       <c r="B92" s="5" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="C92" s="5" t="b">
         <v>0</v>
@@ -5088,19 +5086,19 @@
         <v>0</v>
       </c>
       <c r="E92" s="5" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="F92" s="5">
         <v>9</v>
       </c>
       <c r="G92" s="11">
-        <v>46174</v>
+        <v>46169</v>
       </c>
       <c r="H92" s="11">
-        <v>46185</v>
+        <v>46182</v>
       </c>
       <c r="I92" s="5" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="J92" s="5">
         <v>0</v>
@@ -5126,7 +5124,7 @@
         <v>91</v>
       </c>
       <c r="B93" s="5" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="C93" s="5" t="b">
         <v>0</v>
@@ -5135,20 +5133,20 @@
         <v>0</v>
       </c>
       <c r="E93" s="5" t="s">
+        <v>154</v>
+      </c>
+      <c r="F93" s="5">
+        <v>6</v>
+      </c>
+      <c r="G93" s="11">
+        <v>46174</v>
+      </c>
+      <c r="H93" s="11">
+        <v>46182</v>
+      </c>
+      <c r="I93" s="5" t="s">
         <v>155</v>
       </c>
-      <c r="F93" s="5">
-        <v>8</v>
-      </c>
-      <c r="G93" s="11">
-        <v>46178</v>
-      </c>
-      <c r="H93" s="11">
-        <v>46190</v>
-      </c>
-      <c r="I93" s="5" t="s">
-        <v>156</v>
-      </c>
       <c r="J93" s="5">
         <v>0</v>
       </c>
@@ -5159,13 +5157,13 @@
         <v>0</v>
       </c>
       <c r="M93" s="9">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="N93" s="5" t="s">
         <v>32</v>
       </c>
       <c r="O93" s="9">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="P93" s="0"/>
       <c r="Q93" s="0"/>
@@ -5179,7 +5177,7 @@
         <v>92</v>
       </c>
       <c r="B94" s="5" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="C94" s="5" t="b">
         <v>0</v>
@@ -5188,19 +5186,19 @@
         <v>0</v>
       </c>
       <c r="E94" s="5" t="s">
-        <v>162</v>
+        <v>66</v>
       </c>
       <c r="F94" s="5">
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="G94" s="11">
-        <v>46183</v>
+        <v>46182</v>
       </c>
       <c r="H94" s="11">
-        <v>46199</v>
+        <v>46185</v>
       </c>
       <c r="I94" s="5" t="s">
-        <v>163</v>
+        <v>137</v>
       </c>
       <c r="J94" s="5">
         <v>0</v>
@@ -5211,9 +5209,15 @@
       <c r="L94" s="5">
         <v>0</v>
       </c>
-      <c r="M94" s="0"/>
-      <c r="N94" s="0"/>
-      <c r="O94" s="0"/>
+      <c r="M94" s="9">
+        <v>89</v>
+      </c>
+      <c r="N94" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="O94" s="9">
+        <v>5</v>
+      </c>
       <c r="P94" s="0"/>
       <c r="Q94" s="0"/>
       <c r="R94" s="0"/>
@@ -5226,7 +5230,7 @@
         <v>93</v>
       </c>
       <c r="B95" s="5" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="C95" s="5" t="b">
         <v>0</v>
@@ -5234,21 +5238,17 @@
       <c r="D95" s="9">
         <v>0</v>
       </c>
-      <c r="E95" s="5" t="s">
-        <v>168</v>
-      </c>
+      <c r="E95" s="0"/>
       <c r="F95" s="5">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G95" s="11">
-        <v>46195</v>
+        <v>46182</v>
       </c>
       <c r="H95" s="11">
-        <v>46197</v>
-      </c>
-      <c r="I95" s="5" t="s">
-        <v>24</v>
-      </c>
+        <v>46185</v>
+      </c>
+      <c r="I95" s="0"/>
       <c r="J95" s="5">
         <v>0</v>
       </c>
@@ -5259,13 +5259,13 @@
         <v>0</v>
       </c>
       <c r="M95" s="9">
-        <v>91</v>
+        <v>85</v>
       </c>
       <c r="N95" s="5" t="s">
         <v>32</v>
       </c>
       <c r="O95" s="9">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="P95" s="0"/>
       <c r="Q95" s="0"/>
@@ -5288,19 +5288,19 @@
         <v>0</v>
       </c>
       <c r="E96" s="5" t="s">
-        <v>66</v>
+        <v>171</v>
       </c>
       <c r="F96" s="5">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G96" s="11">
-        <v>46198</v>
+        <v>46188</v>
       </c>
       <c r="H96" s="11">
-        <v>46204</v>
+        <v>46190</v>
       </c>
       <c r="I96" s="5" t="s">
-        <v>137</v>
+        <v>24</v>
       </c>
       <c r="J96" s="5">
         <v>0</v>
@@ -5312,13 +5312,13 @@
         <v>0</v>
       </c>
       <c r="M96" s="9">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="N96" s="5" t="s">
         <v>32</v>
       </c>
       <c r="O96" s="9">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="P96" s="0"/>
       <c r="Q96" s="0"/>
@@ -5332,7 +5332,7 @@
         <v>95</v>
       </c>
       <c r="B97" s="5" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="C97" s="5" t="b">
         <v>0</v>
@@ -5341,19 +5341,19 @@
         <v>0</v>
       </c>
       <c r="E97" s="5" t="s">
-        <v>66</v>
+        <v>163</v>
       </c>
       <c r="F97" s="5">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="G97" s="11">
-        <v>46202</v>
+        <v>46191</v>
       </c>
       <c r="H97" s="11">
         <v>46204</v>
       </c>
       <c r="I97" s="5" t="s">
-        <v>137</v>
+        <v>164</v>
       </c>
       <c r="J97" s="5">
         <v>0</v>
@@ -5371,7 +5371,7 @@
         <v>32</v>
       </c>
       <c r="O97" s="9">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="P97" s="0"/>
       <c r="Q97" s="0"/>
@@ -5385,7 +5385,7 @@
         <v>96</v>
       </c>
       <c r="B98" s="5" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="C98" s="5" t="b">
         <v>0</v>
@@ -5394,19 +5394,19 @@
         <v>0</v>
       </c>
       <c r="E98" s="5" t="s">
-        <v>35</v>
+        <v>171</v>
       </c>
       <c r="F98" s="5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G98" s="11">
-        <v>46202</v>
+        <v>46204</v>
       </c>
       <c r="H98" s="11">
-        <v>46203</v>
+        <v>46204</v>
       </c>
       <c r="I98" s="5" t="s">
-        <v>134</v>
+        <v>24</v>
       </c>
       <c r="J98" s="5">
         <v>0</v>
@@ -5417,9 +5417,15 @@
       <c r="L98" s="5">
         <v>0</v>
       </c>
-      <c r="M98" s="0"/>
-      <c r="N98" s="0"/>
-      <c r="O98" s="0"/>
+      <c r="M98" s="9">
+        <v>94</v>
+      </c>
+      <c r="N98" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="O98" s="9">
+        <v>9</v>
+      </c>
       <c r="P98" s="0"/>
       <c r="Q98" s="0"/>
       <c r="R98" s="0"/>
@@ -5432,7 +5438,7 @@
         <v>97</v>
       </c>
       <c r="B99" s="5" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="C99" s="5" t="b">
         <v>0</v>
@@ -5441,19 +5447,19 @@
         <v>0</v>
       </c>
       <c r="E99" s="5" t="s">
-        <v>176</v>
+        <v>66</v>
       </c>
       <c r="F99" s="5">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G99" s="11">
-        <v>46203</v>
+        <v>46204</v>
       </c>
       <c r="H99" s="11">
         <v>46205</v>
       </c>
       <c r="I99" s="5" t="s">
-        <v>24</v>
+        <v>137</v>
       </c>
       <c r="J99" s="5">
         <v>0</v>
@@ -5465,13 +5471,13 @@
         <v>0</v>
       </c>
       <c r="M99" s="9">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="N99" s="5" t="s">
         <v>32</v>
       </c>
       <c r="O99" s="9">
-        <v>8</v>
+        <v>-1</v>
       </c>
       <c r="P99" s="0"/>
       <c r="Q99" s="0"/>
@@ -5485,7 +5491,7 @@
         <v>98</v>
       </c>
       <c r="B100" s="5" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="C100" s="5" t="b">
         <v>0</v>
@@ -5497,16 +5503,16 @@
         <v>35</v>
       </c>
       <c r="F100" s="5">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G100" s="11">
-        <v>46204</v>
+        <v>46205</v>
       </c>
       <c r="H100" s="11">
-        <v>46206</v>
+        <v>46210</v>
       </c>
       <c r="I100" s="5" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="J100" s="5">
         <v>0</v>
@@ -5532,7 +5538,7 @@
         <v>99</v>
       </c>
       <c r="B101" s="5" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="C101" s="5" t="b">
         <v>0</v>
@@ -5541,19 +5547,19 @@
         <v>0</v>
       </c>
       <c r="E101" s="5" t="s">
-        <v>57</v>
+        <v>35</v>
       </c>
       <c r="F101" s="5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G101" s="11">
-        <v>46209</v>
+        <v>46205</v>
       </c>
       <c r="H101" s="11">
-        <v>46209</v>
+        <v>46206</v>
       </c>
       <c r="I101" s="5" t="s">
-        <v>29</v>
+        <v>134</v>
       </c>
       <c r="J101" s="5">
         <v>0</v>
@@ -5564,15 +5570,9 @@
       <c r="L101" s="5">
         <v>0</v>
       </c>
-      <c r="M101" s="9">
-        <v>98</v>
-      </c>
-      <c r="N101" s="5" t="s">
-        <v>32</v>
-      </c>
-      <c r="O101" s="9">
-        <v>0</v>
-      </c>
+      <c r="M101" s="0"/>
+      <c r="N101" s="0"/>
+      <c r="O101" s="0"/>
       <c r="P101" s="0"/>
       <c r="Q101" s="0"/>
       <c r="R101" s="0"/>
@@ -5585,7 +5585,7 @@
         <v>100</v>
       </c>
       <c r="B102" s="5" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="C102" s="5" t="b">
         <v>0</v>
@@ -5597,16 +5597,16 @@
         <v>35</v>
       </c>
       <c r="F102" s="5">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G102" s="11">
-        <v>46211</v>
+        <v>46205</v>
       </c>
       <c r="H102" s="11">
-        <v>46216</v>
+        <v>46209</v>
       </c>
       <c r="I102" s="5" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="J102" s="5">
         <v>0</v>
@@ -5632,7 +5632,7 @@
         <v>101</v>
       </c>
       <c r="B103" s="5" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="C103" s="5" t="b">
         <v>0</v>
@@ -5641,19 +5641,19 @@
         <v>0</v>
       </c>
       <c r="E103" s="5" t="s">
-        <v>168</v>
+        <v>184</v>
       </c>
       <c r="F103" s="5">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G103" s="11">
-        <v>46211</v>
+        <v>46205</v>
       </c>
       <c r="H103" s="11">
-        <v>46216</v>
+        <v>46206</v>
       </c>
       <c r="I103" s="5" t="s">
-        <v>24</v>
+        <v>185</v>
       </c>
       <c r="J103" s="5">
         <v>0</v>
@@ -5665,17 +5665,23 @@
         <v>0</v>
       </c>
       <c r="M103" s="9">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="N103" s="5" t="s">
         <v>32</v>
       </c>
       <c r="O103" s="9">
-        <v>1</v>
-      </c>
-      <c r="P103" s="0"/>
-      <c r="Q103" s="0"/>
-      <c r="R103" s="0"/>
+        <v>0</v>
+      </c>
+      <c r="P103" s="9">
+        <v>95</v>
+      </c>
+      <c r="Q103" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="R103" s="9">
+        <v>0</v>
+      </c>
       <c r="S103" s="0"/>
       <c r="T103" s="0"/>
       <c r="U103" s="0"/>
@@ -5685,7 +5691,7 @@
         <v>102</v>
       </c>
       <c r="B104" s="5" t="s">
-        <v>183</v>
+        <v>187</v>
       </c>
       <c r="C104" s="5" t="b">
         <v>0</v>
@@ -5694,19 +5700,19 @@
         <v>0</v>
       </c>
       <c r="E104" s="5" t="s">
-        <v>107</v>
+        <v>57</v>
       </c>
       <c r="F104" s="5">
         <v>1</v>
       </c>
       <c r="G104" s="11">
-        <v>46218</v>
+        <v>46210</v>
       </c>
       <c r="H104" s="11">
-        <v>46218</v>
+        <v>46210</v>
       </c>
       <c r="I104" s="5" t="s">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="J104" s="5">
         <v>0</v>
@@ -5718,13 +5724,13 @@
         <v>0</v>
       </c>
       <c r="M104" s="9">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="N104" s="5" t="s">
         <v>32</v>
       </c>
       <c r="O104" s="9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P104" s="0"/>
       <c r="Q104" s="0"/>
@@ -5738,7 +5744,7 @@
         <v>103</v>
       </c>
       <c r="B105" s="5" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="C105" s="5" t="b">
         <v>0</v>
@@ -5747,16 +5753,16 @@
         <v>0</v>
       </c>
       <c r="E105" s="5" t="s">
-        <v>176</v>
+        <v>161</v>
       </c>
       <c r="F105" s="5">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G105" s="11">
-        <v>46219</v>
+        <v>46212</v>
       </c>
       <c r="H105" s="11">
-        <v>46219</v>
+        <v>46217</v>
       </c>
       <c r="I105" s="5" t="s">
         <v>24</v>
@@ -5771,13 +5777,13 @@
         <v>0</v>
       </c>
       <c r="M105" s="9">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="N105" s="5" t="s">
         <v>32</v>
       </c>
       <c r="O105" s="9">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="P105" s="0"/>
       <c r="Q105" s="0"/>
@@ -5791,7 +5797,7 @@
         <v>104</v>
       </c>
       <c r="B106" s="5" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="C106" s="5" t="b">
         <v>0</v>
@@ -5800,16 +5806,16 @@
         <v>0</v>
       </c>
       <c r="E106" s="5" t="s">
-        <v>189</v>
+        <v>107</v>
       </c>
       <c r="F106" s="5">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G106" s="11">
         <v>46219</v>
       </c>
       <c r="H106" s="11">
-        <v>46224</v>
+        <v>46219</v>
       </c>
       <c r="I106" s="5" t="s">
         <v>24</v>
@@ -5824,13 +5830,13 @@
         <v>0</v>
       </c>
       <c r="M106" s="9">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="N106" s="5" t="s">
         <v>32</v>
       </c>
       <c r="O106" s="9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P106" s="0"/>
       <c r="Q106" s="0"/>
@@ -5844,7 +5850,7 @@
         <v>105</v>
       </c>
       <c r="B107" s="5" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="C107" s="5" t="b">
         <v>0</v>
@@ -5853,16 +5859,16 @@
         <v>0</v>
       </c>
       <c r="E107" s="5" t="s">
-        <v>57</v>
+        <v>193</v>
       </c>
       <c r="F107" s="5">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G107" s="11">
         <v>46220</v>
       </c>
       <c r="H107" s="11">
-        <v>46223</v>
+        <v>46225</v>
       </c>
       <c r="I107" s="5" t="s">
         <v>24</v>
@@ -5877,13 +5883,13 @@
         <v>0</v>
       </c>
       <c r="M107" s="9">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="N107" s="5" t="s">
         <v>32</v>
       </c>
       <c r="O107" s="9">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="P107" s="0"/>
       <c r="Q107" s="0"/>
@@ -5897,7 +5903,7 @@
         <v>106</v>
       </c>
       <c r="B108" s="5" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="C108" s="5" t="b">
         <v>0</v>
@@ -5906,19 +5912,19 @@
         <v>0</v>
       </c>
       <c r="E108" s="5" t="s">
-        <v>193</v>
+        <v>57</v>
       </c>
       <c r="F108" s="5">
         <v>2</v>
       </c>
       <c r="G108" s="11">
-        <v>46220</v>
+        <v>46223</v>
       </c>
       <c r="H108" s="11">
-        <v>46223</v>
+        <v>46224</v>
       </c>
       <c r="I108" s="5" t="s">
-        <v>194</v>
+        <v>24</v>
       </c>
       <c r="J108" s="5">
         <v>0</v>
@@ -5936,17 +5942,11 @@
         <v>32</v>
       </c>
       <c r="O108" s="9">
-        <v>0</v>
-      </c>
-      <c r="P108" s="9">
-        <v>92</v>
-      </c>
-      <c r="Q108" s="5" t="s">
-        <v>32</v>
-      </c>
-      <c r="R108" s="9">
-        <v>0</v>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="P108" s="0"/>
+      <c r="Q108" s="0"/>
+      <c r="R108" s="0"/>
       <c r="S108" s="0"/>
       <c r="T108" s="0"/>
       <c r="U108" s="0"/>
@@ -5971,10 +5971,10 @@
         <v>1</v>
       </c>
       <c r="G109" s="11">
-        <v>46225</v>
+        <v>46226</v>
       </c>
       <c r="H109" s="11">
-        <v>46225</v>
+        <v>46226</v>
       </c>
       <c r="I109" s="5" t="s">
         <v>24</v>
@@ -5989,7 +5989,7 @@
         <v>0</v>
       </c>
       <c r="M109" s="9">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="N109" s="5" t="s">
         <v>32</v>
@@ -6022,10 +6022,10 @@
         <v>41</v>
       </c>
       <c r="G110" s="11">
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="H110" s="11">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="I110" s="0"/>
       <c r="J110" s="5">

</xml_diff>